<commit_message>
Update legacy xls-to-xlsx conversion worker and Excel utilities
- Improve LegacyXlsClassLoader and HssfToXssf handling in the isolated
  legacy-xls-worker JAR
- Update LegacyXlsTransformWorker and rebuild legacy-xls-worker.jar
- Adjust ExcelUtilSerImp and jxlcompat.Cell for the updated worker
- Update generated template/output xlsx samples

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WebRoot/resources/template/HTSV/MassNewAction_Hire.xlsx
+++ b/WebRoot/resources/template/HTSV/MassNewAction_Hire.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Java\WorkSpace\Hanwha_HTSV\WebRoot\resources\template\HTSV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA28ABB8-30B8-4E4B-8765-677E00A79175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD425CBE-5552-45AA-804F-3188C9D34FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="3075" windowWidth="38700" windowHeight="15225" xr2:uid="{6845AF8B-A828-4AC5-BFAD-A0B0D0069EB3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{6845AF8B-A828-4AC5-BFAD-A0B0D0069EB3}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="65">
   <si>
     <t>Red font: you must enter a project</t>
   </si>
@@ -540,7 +540,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="186" formatCode="yyyymmdd"/>
+    <numFmt numFmtId="164" formatCode="yyyymmdd"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -745,10 +745,10 @@
     <xf numFmtId="49" fontId="14" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="186" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="186" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -763,10 +763,10 @@
     <xf numFmtId="49" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1671,9 +1671,7 @@
       <c r="D7" s="14"/>
       <c r="E7" s="13"/>
       <c r="F7" s="14"/>
-      <c r="G7" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G7" s="13"/>
       <c r="H7" s="15" t="str">
         <f>IF(G7="","",VLOOKUP(G7,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -1843,9 +1841,7 @@
       <c r="F8" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G8" s="13"/>
       <c r="H8" s="15" t="str">
         <f>IF(G8="","",VLOOKUP(G8,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -2029,9 +2025,7 @@
       <c r="F9" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G9" s="13"/>
       <c r="H9" s="15" t="str">
         <f>IF(G9="","",VLOOKUP(G9,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -2215,9 +2209,7 @@
       <c r="F10" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G10" s="13"/>
       <c r="H10" s="15" t="str">
         <f>IF(G10="","",VLOOKUP(G10,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -2401,9 +2393,7 @@
       <c r="F11" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G11" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G11" s="13"/>
       <c r="H11" s="15" t="str">
         <f>IF(G11="","",VLOOKUP(G11,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -2587,9 +2577,7 @@
       <c r="F12" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G12" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G12" s="13"/>
       <c r="H12" s="15" t="str">
         <f>IF(G12="","",VLOOKUP(G12,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -2773,9 +2761,7 @@
       <c r="F13" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G13" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G13" s="13"/>
       <c r="H13" s="15" t="str">
         <f>IF(G13="","",VLOOKUP(G13,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -2959,9 +2945,7 @@
       <c r="F14" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G14" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G14" s="13"/>
       <c r="H14" s="15" t="str">
         <f>IF(G14="","",VLOOKUP(G14,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -3145,9 +3129,7 @@
       <c r="F15" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G15" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G15" s="13"/>
       <c r="H15" s="15" t="str">
         <f>IF(G15="","",VLOOKUP(G15,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -3331,9 +3313,7 @@
       <c r="F16" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="G16" s="13"/>
       <c r="H16" s="15" t="str">
         <f>IF(G16="","",VLOOKUP(G16,TemplateCode!$A$2:$C$450,2,FALSE))</f>
         <v/>
@@ -3510,7 +3490,7 @@
     <mergeCell ref="A4:G4"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
-  <dataValidations count="16">
+  <dataValidations count="15">
     <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A7:B16 E7:E16" xr:uid="{106FCC2C-2FD5-41DB-B376-C4B9EAD7EBE2}">
       <formula1>256</formula1>
     </dataValidation>
@@ -3541,7 +3521,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE7:AE16" xr:uid="{7038CB83-FDB7-47EF-8A02-8C503543E2DC}">
       <formula1>zzxl</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN8:AN16" xr:uid="{0F279B33-E719-4EFC-8CD7-28D03ED7A3B4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN7:AN16" xr:uid="{0F279B33-E719-4EFC-8CD7-28D03ED7A3B4}">
       <formula1>xb</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AQ7:AQ16" xr:uid="{9AAC8BC8-6DF0-47B0-BEB3-006FFE76C6E4}">
@@ -3552,9 +3532,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AX7:AX16" xr:uid="{F5DCBFB8-9E10-415D-8E63-BF2774EEDF41}">
       <formula1>jhqf</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN7" xr:uid="{48AB9151-9CC4-4B17-814F-9CAA86FE1341}">
-      <formula1>xb</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB7:AB16" xr:uid="{7B46F606-5DF9-436B-B765-1954C596AE07}">
       <formula1>zq</formula1>
@@ -3850,6 +3827,12 @@
     <row r="208" ht="12.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="U1:W1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="Q1:S1"/>
     <mergeCell ref="AW1:AY1"/>
     <mergeCell ref="Y1:AA1"/>
     <mergeCell ref="AC1:AE1"/>
@@ -3857,12 +3840,6 @@
     <mergeCell ref="AK1:AM1"/>
     <mergeCell ref="AO1:AQ1"/>
     <mergeCell ref="AS1:AU1"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="Q1:S1"/>
-    <mergeCell ref="U1:W1"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>